<commit_message>
Agregar códigos de barras y SKU a la remisión Tienda Oct 20
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014X9aKeEEzv3fy6HSjYT7Md
</commit_message>
<xml_diff>
--- a/remisiones/Remision_Tienda_Oct20_2026.xlsx
+++ b/remisiones/Remision_Tienda_Oct20_2026.xlsx
@@ -87,14 +87,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -464,15 +467,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,12 +493,12 @@
           <t>Lobster Mini</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Fecha:</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
@@ -505,12 +510,12 @@
           <t>Destino: Tienda</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>No.:</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -520,25 +525,35 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>Código de barras</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>Producto</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Talla</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Precio unitario</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
@@ -548,24 +563,34 @@
       <c r="A6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>610735448</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>FAL-CHERRY-4T</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Falda Tejida Cherry Playful</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>4T</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="5" t="n">
         <v>139900</v>
       </c>
-      <c r="F6" s="4">
-        <f>D6*E6</f>
+      <c r="H6" s="5">
+        <f>F6*G6</f>
         <v/>
       </c>
     </row>
@@ -573,24 +598,34 @@
       <c r="A7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>407058324</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>LEG-CANCHEROS-4T</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Leggings Cancheros</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>4T</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="5" t="n">
         <v>98900</v>
       </c>
-      <c r="F7" s="4">
-        <f>D7*E7</f>
+      <c r="H7" s="5">
+        <f>F7*G7</f>
         <v/>
       </c>
     </row>
@@ -598,24 +633,34 @@
       <c r="A8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>52162361</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>CAM-PLUM-10</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Camiseta Retro Plum</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>10T</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="n">
         <v>89900</v>
       </c>
-      <c r="F8" s="4">
-        <f>D8*E8</f>
+      <c r="H8" s="5">
+        <f>F8*G8</f>
         <v/>
       </c>
     </row>
@@ -623,24 +668,34 @@
       <c r="A9" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>925650046</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>BUZ-CHERRY-10</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Buzo Cherry Kick</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>10T</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="5" t="n">
         <v>139900</v>
       </c>
-      <c r="F9" s="4">
-        <f>D9*E9</f>
+      <c r="H9" s="5">
+        <f>F9*G9</f>
         <v/>
       </c>
     </row>
@@ -648,22 +703,24 @@
       <c r="A10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Camiseta Barcos</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>7-8T</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="4">
-        <f>D10*E10</f>
+      <c r="F10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="5">
+        <f>F10*G10</f>
         <v/>
       </c>
     </row>
@@ -671,22 +728,24 @@
       <c r="A11" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Camiseta Favorite Place</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>6T</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="4">
-        <f>D11*E11</f>
+      <c r="F11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="5">
+        <f>F11*G11</f>
         <v/>
       </c>
     </row>
@@ -694,22 +753,24 @@
       <c r="A12" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Camiseta Mixer Azul Espacial</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>5T</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="4">
-        <f>D12*E12</f>
+      <c r="F12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="5">
+        <f>F12*G12</f>
         <v/>
       </c>
     </row>
@@ -717,22 +778,24 @@
       <c r="A13" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Camiseta Mixer Café Explorador</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>4T</t>
         </is>
       </c>
-      <c r="D13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="4">
-        <f>D13*E13</f>
+      <c r="F13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="5">
+        <f>F13*G13</f>
         <v/>
       </c>
     </row>
@@ -740,22 +803,24 @@
       <c r="A14" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Camiseta Mixer Roja Marte</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>2T</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="4">
-        <f>D14*E14</f>
+      <c r="F14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="5">
+        <f>F14*G14</f>
         <v/>
       </c>
     </row>
@@ -763,22 +828,24 @@
       <c r="A15" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Camiseta Mixer Roja Marte</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>4T</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="4">
-        <f>D15*E15</f>
+      <c r="F15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="8" t="n"/>
+      <c r="H15" s="5">
+        <f>F15*G15</f>
         <v/>
       </c>
     </row>
@@ -786,22 +853,24 @@
       <c r="A16" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Camiseta Mixer oso pardo</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>5T</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="4">
-        <f>D16*E16</f>
+      <c r="F16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="5">
+        <f>F16*G16</f>
         <v/>
       </c>
     </row>
@@ -809,22 +878,24 @@
       <c r="A17" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Pijama Formas</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>7-8T</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="4">
-        <f>D17*E17</f>
+      <c r="F17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="5">
+        <f>F17*G17</f>
         <v/>
       </c>
     </row>
@@ -832,22 +903,24 @@
       <c r="A18" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Vestido Croissants</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>5T</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="4">
-        <f>D18*E18</f>
+      <c r="F18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="8" t="n"/>
+      <c r="H18" s="5">
+        <f>F18*G18</f>
         <v/>
       </c>
     </row>
@@ -855,22 +928,24 @@
       <c r="A19" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Vestido Croissants</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>6T</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="4">
-        <f>D19*E19</f>
+      <c r="F19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="8" t="n"/>
+      <c r="H19" s="5">
+        <f>F19*G19</f>
         <v/>
       </c>
     </row>
@@ -878,22 +953,24 @@
       <c r="A20" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Vestido Mantelito</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>5T</t>
         </is>
       </c>
-      <c r="D20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="4">
-        <f>D20*E20</f>
+      <c r="F20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="5">
+        <f>F20*G20</f>
         <v/>
       </c>
     </row>
@@ -901,22 +978,24 @@
       <c r="A21" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Vestido Mantelito</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>6T</t>
         </is>
       </c>
-      <c r="D21" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="4">
-        <f>D21*E21</f>
+      <c r="F21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="8" t="n"/>
+      <c r="H21" s="5">
+        <f>F21*G21</f>
         <v/>
       </c>
     </row>
@@ -924,22 +1003,24 @@
       <c r="A22" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>buzo-trebol</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>6T</t>
         </is>
       </c>
-      <c r="D22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="4">
-        <f>D22*E22</f>
+      <c r="F22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="5">
+        <f>F22*G22</f>
         <v/>
       </c>
     </row>
@@ -947,22 +1028,24 @@
       <c r="A23" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>camiseta-mil-estrellas</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>8T</t>
         </is>
       </c>
-      <c r="D23" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="4">
-        <f>D23*E23</f>
+      <c r="F23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="8" t="n"/>
+      <c r="H23" s="5">
+        <f>F23*G23</f>
         <v/>
       </c>
     </row>
@@ -970,44 +1053,46 @@
       <c r="A24" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>pantalon-trebol</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>4T</t>
         </is>
       </c>
-      <c r="D24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="4">
-        <f>D24*E24</f>
+      <c r="F24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="5">
+        <f>F24*G24</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="6" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D25" s="6">
-        <f>SUM(D6:D24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="7">
+      <c r="F25" s="9">
         <f>SUM(F6:F24)</f>
         <v/>
       </c>
+      <c r="H25" s="10">
+        <f>SUM(H6:H24)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>Celdas amarillas: precio pendiente (producto no encontrado en la tienda Shopify conectada).</t>
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Celdas amarillas: precio / código pendiente (producto no encontrado en la tienda Shopify conectada).</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1102,7 @@
           <t>______________________</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>______________________</t>
         </is>
@@ -1029,7 +1114,7 @@
           <t>Entrega</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Recibe</t>
         </is>

</xml_diff>